<commit_message>
WIP static table prep and join
</commit_message>
<xml_diff>
--- a/static_tables.xlsx
+++ b/static_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26501"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55586\Desktop\Access tool\Python Tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55586\Desktop\tools\access tool\access-tool-migration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF7D51C-B65A-4CF1-8AB9-81FE1B2F1ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF58B70-41FC-4162-A55A-28D98E23A206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12645" yWindow="3210" windowWidth="23040" windowHeight="14820" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11280" yWindow="3270" windowWidth="24060" windowHeight="17160" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_PollutantCrosswalk_andMe" sheetId="1" r:id="rId1"/>
@@ -9197,9 +9197,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -9237,9 +9237,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -9272,26 +9272,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -9324,26 +9307,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -65391,12 +65357,12 @@
   <dimension ref="A1:F135"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.5703125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="44" style="5" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="30.5703125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="5" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>

</xml_diff>